<commit_message>
Changes for HW requests.
</commit_message>
<xml_diff>
--- a/XLSX/ActualOrderAmountOrderBalance.xlsx
+++ b/XLSX/ActualOrderAmountOrderBalance.xlsx
@@ -1,63 +1,65 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
-  <x:workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ShawnLi\Documents\Cals\Hagiwara_Upgrade\BC\AL\Hagiwara\XLSX\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04C4CB2E-9AF3-443E-AACB-A6186488D02C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <x:bookViews>
-    <x:workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </x:bookViews>
-  <x:sheets>
-    <x:sheet name="Date" sheetId="10" r:id="rId1"/>
-    <x:sheet name="Remaining Sales Order" sheetId="11" r:id="rId2"/>
-    <x:sheet name="Sales Order Actual" sheetId="12" r:id="rId3"/>
-    <x:sheet name="Sales Order Balance" sheetId="13" r:id="rId4"/>
-    <x:sheet name="Customer" sheetId="14" r:id="rId5"/>
-    <x:sheet name="TranslationData" sheetId="2" state="hidden" r:id="rId6"/>
-    <x:sheet name="CaptionData" sheetId="3" state="hidden" r:id="rId7"/>
-    <x:sheet name="Aggregated Metadata" sheetId="4" state="hidden" r:id="rId8"/>
-    <x:sheet name="DateSheet" sheetId="5" state="hidden" r:id="rId9"/>
-    <x:sheet name="RemainingSalesOrder" sheetId="6" state="hidden" r:id="rId10"/>
-    <x:sheet name="SalesOrderActual" sheetId="7" state="hidden" r:id="rId11"/>
-    <x:sheet name="SalesOrderBalance" sheetId="8" state="hidden" r:id="rId12"/>
-    <x:sheet name="CustomerSheet" sheetId="9" state="hidden" r:id="rId13"/>
-  </x:sheets>
-  <x:definedNames>
-    <x:definedName name="ReportMetadata.AboutThisReportText" comment="Use this function to get the About This Report Text from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("About This Report Text",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportMetadata.AboutThisReportTitle" comment="Use this function to get the About This Report Title from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("About This Report Title",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportMetadata.ExtensionID" comment="Use this function to get the Extension Id from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension ID",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportMetadata.ExtensionName" comment="Use this function to get the Extension Name from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Name",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportMetadata.ExtensionPublisher" comment="Use this function to get the Extension Publisher from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Publisher",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportMetadata.ExtensionVersion" comment="Use this function to get the Extension Version from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Version",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportMetadata.ObjectCaption" comment="Use this function to get the Object Caption from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object Caption",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportMetadata.ObjectID" comment="Use this function to get the Object ID from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object ID",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportMetadata.ObjectName" comment="Use this function to get the Object Name from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object Name",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportMetadata.ReportHelpLink" comment="Use this function to get the Report help link from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Report help link",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.CompanyDisplayName" comment="Use this function to get the Company Display name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company display name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.CompanyId" comment="Use this function to get the Company Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.CompanyName" comment="Use this function to get the Company name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.Date" comment="Use this function to get the Date from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Date",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.DateLocal" comment="Use this function to get the Date (Local) from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Date (Local)",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.EnvironmentName" comment="Use this function to get the Environment name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Environment name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.EnvironmentType" comment="Use this function to get the Environment type from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Environment type",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.FormatRegion" comment="Use this function to get the Format Region from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Format Region",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.Language" comment="Use this function to get the Language from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Language",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.LayoutCaption" comment="Use this function to get the Layout caption from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout caption",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.LayoutId" comment="Use this function to get the Layout id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.LayoutName" comment="Use this function to get the Layout name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.TenantEntraId" comment="Use this function to get the Tenant Entra Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Entra Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.TenantId" comment="Use this function to get the Tenant Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.UserName" comment="Use this function to get the User name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("User name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-    <x:definedName name="ReportRequest.UTCOffset" comment="Use this function to get the UTC Offset from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("UTC Offset",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
-  </x:definedNames>
-  <x:calcPr calcId="191029"/>
-  <x:extLst>
-    <x:ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED4527C9-C1E9-4199-9487-0DCF79BB0C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="15700" tabRatio="878" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Date" sheetId="11" r:id="rId1"/>
+    <sheet name="Remaining Sales Order" sheetId="12" r:id="rId2"/>
+    <sheet name="Sales Order Actual" sheetId="13" r:id="rId3"/>
+    <sheet name="Sales Order Balance" sheetId="14" r:id="rId4"/>
+    <sheet name="Customer" sheetId="15" r:id="rId5"/>
+    <sheet name="Order Summary by Customer" sheetId="16" r:id="rId6"/>
+    <sheet name="TranslationData" sheetId="2" r:id="rId7"/>
+    <sheet name="CaptionData" sheetId="3" r:id="rId8"/>
+    <sheet name="Aggregated Metadata" sheetId="4" r:id="rId9"/>
+    <sheet name="DateSheet" sheetId="5" r:id="rId10"/>
+    <sheet name="RemainingSalesOrder" sheetId="6" r:id="rId11"/>
+    <sheet name="SalesOrderActual" sheetId="7" r:id="rId12"/>
+    <sheet name="SalesOrderBalance" sheetId="8" r:id="rId13"/>
+    <sheet name="CustomerSheet" sheetId="9" r:id="rId14"/>
+    <sheet name="OrderSummarybyCustomer" sheetId="10" r:id="rId15"/>
+  </sheets>
+  <definedNames>
+    <definedName name="ReportMetadata.AboutThisReportText" comment="Use this function to get the About This Report Text from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("About This Report Text",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportMetadata.AboutThisReportTitle" comment="Use this function to get the About This Report Title from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("About This Report Title",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportMetadata.ExtensionID" comment="Use this function to get the Extension Id from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension ID",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportMetadata.ExtensionName" comment="Use this function to get the Extension Name from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Name",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportMetadata.ExtensionPublisher" comment="Use this function to get the Extension Publisher from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Publisher",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportMetadata.ExtensionVersion" comment="Use this function to get the Extension Version from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Version",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportMetadata.ObjectCaption" comment="Use this function to get the Object Caption from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object Caption",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportMetadata.ObjectID" comment="Use this function to get the Object ID from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object ID",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportMetadata.ObjectName" comment="Use this function to get the Object Name from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object Name",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportMetadata.ReportHelpLink" comment="Use this function to get the Report help link from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Report help link",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.CompanyDisplayName" comment="Use this function to get the Company Display name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company display name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.CompanyId" comment="Use this function to get the Company Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.CompanyName" comment="Use this function to get the Company name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.Date" comment="Use this function to get the Date from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Date",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.DateLocal" comment="Use this function to get the Date (Local) from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Date (Local)",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.EnvironmentName" comment="Use this function to get the Environment name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Environment name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.EnvironmentType" comment="Use this function to get the Environment type from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Environment type",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.FormatRegion" comment="Use this function to get the Format Region from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Format Region",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.Language" comment="Use this function to get the Language from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Language",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.LayoutCaption" comment="Use this function to get the Layout caption from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout caption",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.LayoutId" comment="Use this function to get the Layout id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.LayoutName" comment="Use this function to get the Layout name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.TenantEntraId" comment="Use this function to get the Tenant Entra Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Entra Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.TenantId" comment="Use this function to get the Tenant Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.UserName" comment="Use this function to get the User name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("User name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+    <definedName name="ReportRequest.UTCOffset" comment="Use this function to get the UTC Offset from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("UTC Offset",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
@@ -67,13 +69,13 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </x:ext>
-  </x:extLst>
-</x:workbook>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -95,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="224">
   <si>
     <t>Language</t>
   </si>
@@ -295,6 +297,12 @@
     <t>To</t>
   </si>
   <si>
+    <t>CustPostGrpFilter</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>SO_DocumentType</t>
   </si>
   <si>
@@ -397,9 +405,6 @@
     <t>SO_ApprovedAmount</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>False</t>
   </si>
   <si>
@@ -571,6 +576,18 @@
     <t>CU_ShippingAgentCode</t>
   </si>
   <si>
+    <t>Sum_No</t>
+  </si>
+  <si>
+    <t>Sum_Name</t>
+  </si>
+  <si>
+    <t>Sum_ActOrdAmount</t>
+  </si>
+  <si>
+    <t>Sum_OrdBalance</t>
+  </si>
+  <si>
     <t>Document Type</t>
   </si>
   <si>
@@ -662,78 +679,6 @@
   </si>
   <si>
     <t>Customer Posting Group</t>
-  </si>
-  <si>
-    <t>Posting Date</t>
-  </si>
-  <si>
-    <t>Document Date</t>
-  </si>
-  <si>
-    <t>Customer No.</t>
-  </si>
-  <si>
-    <t>Customer</t>
-  </si>
-  <si>
-    <t>Order No.</t>
-  </si>
-  <si>
-    <t>OEM Name</t>
-  </si>
-  <si>
-    <t>Currency Code</t>
-  </si>
-  <si>
-    <t>Due Date</t>
-  </si>
-  <si>
-    <t>Amount</t>
-  </si>
-  <si>
-    <t>Amount LCY</t>
-  </si>
-  <si>
-    <t>Amount Including VAT</t>
-  </si>
-  <si>
-    <t>External Document No.</t>
-  </si>
-  <si>
-    <t>Remaining Amount</t>
-  </si>
-  <si>
-    <t>No. Printed</t>
-  </si>
-  <si>
-    <t>Closed</t>
-  </si>
-  <si>
-    <t>Cancelled</t>
-  </si>
-  <si>
-    <t>Corrective</t>
-  </si>
-  <si>
-    <t>Shipment Method Code</t>
-  </si>
-  <si>
-    <t>Customer group Code</t>
-  </si>
-  <si>
-    <t>Familiar Name</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Country/Region Code</t>
-  </si>
-  <si>
-    <t>County</t>
-  </si>
-  <si>
-    <t>Shipping Agent Code</t>
   </si>
   <si>
     <t>Approved Quantity</t>
@@ -745,6 +690,88 @@
   </si>
   <si>
     <t>Approved Amount Excl. VAT</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Posting Date</t>
+  </si>
+  <si>
+    <t>Document Date</t>
+  </si>
+  <si>
+    <t>Customer No.</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>Order No.</t>
+  </si>
+  <si>
+    <t>OEM Name</t>
+  </si>
+  <si>
+    <t>Currency Code</t>
+  </si>
+  <si>
+    <t>Due Date</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Amount LCY</t>
+  </si>
+  <si>
+    <t>Amount Including VAT</t>
+  </si>
+  <si>
+    <t>External Document No.</t>
+  </si>
+  <si>
+    <t>Remaining Amount</t>
+  </si>
+  <si>
+    <t>No. Printed</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>Cancelled</t>
+  </si>
+  <si>
+    <t>Corrective</t>
+  </si>
+  <si>
+    <t>Shipment Method Code</t>
+  </si>
+  <si>
+    <t>Customer group Code</t>
+  </si>
+  <si>
+    <t>Familiar Name</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Country/Region Code</t>
+  </si>
+  <si>
+    <t>County</t>
+  </si>
+  <si>
+    <t>Shipping Agent Code</t>
+  </si>
+  <si>
+    <t>Actual Order Amount</t>
+  </si>
+  <si>
+    <t>Order Balance</t>
+  </si>
+  <si>
+    <t>Customer Posting Group</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -835,7 +862,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="14">
     <dxf>
       <fill>
         <patternFill>
@@ -861,6 +888,31 @@
       <fill>
         <patternFill>
           <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC0C0C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1115,53 +1167,66 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="SalesOrderBalance" displayName="SalesOrderBalance" ref="A1:X2" totalsRowShown="0" headerRowDxfId="5" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" mc:Ignorable="xr xr3">
-  <x:autoFilter ref="A1:X2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
-  <x:tableColumns count="24">
-    <x:tableColumn id="1" name="BAL_ShipmentDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="2" name="BAL_PostingDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="3" name="BAL_DocumentDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="4" name="BAL_No" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="5" name="BAL_CustomerNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="6" name="BAL_Customer" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="7" name="BAL_OrderNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="8" name="BAL_OEMNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="9" name="BAL_OEMName" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="10" name="BAL_CurrencyCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="11" name="BAL_DueDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="12" name="BAL_Amount" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="13" name="BAL_AmountLCY" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="14" name="BAL_AmountIncludingVAT" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="15" name="BAL_ExternalDocumentNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="16" name="BAL_RemainingAmount" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="17" name="BAL_LocationCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="18" name="BAL_PrintedNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="19" name="BAL_Closed" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="20" name="BAL_Cancelled" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="21" name="BAL_Corrective" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="22" name="BAL_ShipmentMethodCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="23" name="BAL_CustomerGroupCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="24" name="BAL_CustomerPostingGroup" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="SalesOrderBalance" displayName="SalesOrderBalance" ref="A1:X2" totalsRowShown="0" headerRowDxfId="6">
+  <autoFilter ref="A1:X2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
+  <tableColumns count="24">
+    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_ShipmentDate"/>
+    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_PostingDate"/>
+    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_DocumentDate"/>
+    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_No"/>
+    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_CustomerNo"/>
+    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_Customer"/>
+    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_OrderNo"/>
+    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_OEMNo"/>
+    <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_OEMName"/>
+    <tableColumn id="10" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_CurrencyCode"/>
+    <tableColumn id="11" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_DueDate"/>
+    <tableColumn id="12" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_Amount"/>
+    <tableColumn id="13" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_AmountLCY"/>
+    <tableColumn id="14" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_AmountIncludingVAT"/>
+    <tableColumn id="15" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_ExternalDocumentNo"/>
+    <tableColumn id="16" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_RemainingAmount"/>
+    <tableColumn id="17" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_LocationCode"/>
+    <tableColumn id="18" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_PrintedNo"/>
+    <tableColumn id="19" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_Closed"/>
+    <tableColumn id="20" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_Cancelled"/>
+    <tableColumn id="21" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_Corrective"/>
+    <tableColumn id="22" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_ShipmentMethodCode"/>
+    <tableColumn id="23" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_CustomerGroupCode"/>
+    <tableColumn id="24" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="BAL_CustomerPostingGroup"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="CustomerSheet" displayName="CustomerSheet" ref="A1:H2" totalsRowShown="0" headerRowDxfId="4" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" mc:Ignorable="xr xr3">
-  <x:autoFilter ref="A1:H2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
-  <x:tableColumns count="8">
-    <x:tableColumn id="1" name="CU_No" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="2" name="CU_FamiliarName" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="3" name="CU_Name" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="4" name="CU_CountryRegionCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="5" name="CU_County" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="6" name="CU_CustomerPostingGroup" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="7" name="CU_ShipmentMethodCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="8" name="CU_ShippingAgentCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="CustomerSheet" displayName="CustomerSheet" ref="A1:H2" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:H2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="CU_No"/>
+    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="CU_FamiliarName"/>
+    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="CU_Name"/>
+    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="CU_CountryRegionCode"/>
+    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="CU_County"/>
+    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="CU_CustomerPostingGroup"/>
+    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="CU_ShipmentMethodCode"/>
+    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="CU_ShippingAgentCode"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="OrderSummarybyCustomer" displayName="OrderSummarybyCustomer" ref="A1:D2" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:D2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Sum_No"/>
+    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Sum_Name"/>
+    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Sum_ActOrdAmount"/>
+    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Sum_OrdBalance"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1176,7 +1241,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{134EB915-8B19-4838-BDED-CECBACACF4F9}" name="ReportMetadataValues" displayName="ReportMetadataValues" ref="A1:B11" totalsRowShown="0" headerRowDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{134EB915-8B19-4838-BDED-CECBACACF4F9}" name="ReportMetadataValues" displayName="ReportMetadataValues" ref="A1:B11" totalsRowShown="0" headerRowDxfId="13">
   <autoFilter ref="A1:B11" xr:uid="{134EB915-8B19-4838-BDED-CECBACACF4F9}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{5CBC1C08-5A8D-42BB-92CA-C3F1D0EF0A4D}" name="Report Property"/>
@@ -1187,7 +1252,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1DFF5EE2-2A86-40DE-9DFD-1E96553323F6}" name="ReportRequestValues" displayName="ReportRequestValues" ref="D1:E17" totalsRowShown="0" headerRowDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1DFF5EE2-2A86-40DE-9DFD-1E96553323F6}" name="ReportRequestValues" displayName="ReportRequestValues" ref="D1:E17" totalsRowShown="0" headerRowDxfId="12">
   <autoFilter ref="D1:E17" xr:uid="{1DFF5EE2-2A86-40DE-9DFD-1E96553323F6}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{E6EF2D44-8AB2-42E8-A7E3-9B148922AA59}" name="Request Property"/>
@@ -1198,7 +1263,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{8D3A40BA-47FA-41F3-82A4-C5BD4909C0B4}" name="ReportRequestPageValues" displayName="ReportRequestPageValues" ref="G1:H2" totalsRowShown="0" headerRowDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{8D3A40BA-47FA-41F3-82A4-C5BD4909C0B4}" name="ReportRequestPageValues" displayName="ReportRequestPageValues" ref="G1:H2" totalsRowShown="0" headerRowDxfId="11">
   <autoFilter ref="G1:H2" xr:uid="{8D3A40BA-47FA-41F3-82A4-C5BD4909C0B4}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{023648B2-C225-4580-B767-C48467418032}" name="Request Page Option"/>
@@ -1209,7 +1274,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D269260C-C433-478B-84A3-3CB73C333872}" name="ReportFilterValues" displayName="ReportFilterValues" ref="J1:K2" totalsRowShown="0" headerRowDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D269260C-C433-478B-84A3-3CB73C333872}" name="ReportFilterValues" displayName="ReportFilterValues" ref="J1:K2" totalsRowShown="0" headerRowDxfId="10">
   <autoFilter ref="J1:K2" xr:uid="{D269260C-C433-478B-84A3-3CB73C333872}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D710F0AA-F8F4-4DB2-BC43-E65C2054A321}" name="Filter"/>
@@ -1220,90 +1285,91 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DateSheet" displayName="DateSheet" ref="A1:B2" totalsRowShown="0" headerRowDxfId="8" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" mc:Ignorable="xr xr3">
-  <x:autoFilter ref="A1:B2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
-  <x:tableColumns count="2">
-    <x:tableColumn id="1" name="From" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="2" name="To" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="DateSheet" displayName="DateSheet" ref="A1:C2" totalsRowShown="0" headerRowDxfId="9">
+  <autoFilter ref="A1:C2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="From"/>
+    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="To"/>
+    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="CustPostGrpFilter"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="RemainingSalesOrder" displayName="RemainingSalesOrder" ref="A1:AH2" totalsRowShown="0" headerRowDxfId="7" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" mc:Ignorable="xr xr3">
-  <x:autoFilter ref="A1:AH2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
-  <x:tableColumns count="34">
-    <x:tableColumn id="1" name="SO_DocumentType" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="2" name="SO_DocumentNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="3" name="SO_SelltoCustomerNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="4" name="SO_Type" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="5" name="SO_No" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="6" name="SO_CustomerItemNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="7" name="SO_PartsNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="8" name="SO_Rank" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="9" name="SO_Products" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="10" name="SO_OEMNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="11" name="SO_OrderDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="12" name="SO_PromisedDeliveryDate1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="13" name="SO_RequestedDeliveryDate1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="14" name="SO_Description" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="15" name="SO_CustomerOrderNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="16" name="SO_LocationCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="17" name="SO_Reserve" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="18" name="SO_Quantity" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="19" name="SO_ReservedQtyBase" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="20" name="SO_FullyReserved" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="21" name="SO_UnitofMeasureCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="22" name="SO_UnitPriceExcl_VAT" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="23" name="SO_UnitCost" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="24" name="SO_UnitCost_LCY" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="25" name="SO_LineAmountExclVAT" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="26" name="SO_LineAmountExclVATLCY" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="27" name="SO_ShipmentDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="28" name="SO_OutstandingQuantity" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="29" name="SO_OutstandingQtyBase" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="30" name="SO_Calculated" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="31" name="SO_CustomerPostingGroup" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="32" name="SO_ApprovedQuantity" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="33" name="SO_ApprovedUnitPrice" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="34" name="SO_ApprovedAmount" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="RemainingSalesOrder" displayName="RemainingSalesOrder" ref="A1:AH2" totalsRowShown="0" headerRowDxfId="8">
+  <autoFilter ref="A1:AH2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
+  <tableColumns count="34">
+    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_DocumentType"/>
+    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_DocumentNo"/>
+    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_SelltoCustomerNo"/>
+    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_Type"/>
+    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_No"/>
+    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_CustomerItemNo"/>
+    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_PartsNo"/>
+    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_Rank"/>
+    <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_Products"/>
+    <tableColumn id="10" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_OEMNo"/>
+    <tableColumn id="11" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_OrderDate"/>
+    <tableColumn id="12" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_PromisedDeliveryDate1"/>
+    <tableColumn id="13" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_RequestedDeliveryDate1"/>
+    <tableColumn id="14" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_Description"/>
+    <tableColumn id="15" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_CustomerOrderNo"/>
+    <tableColumn id="16" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_LocationCode"/>
+    <tableColumn id="17" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_Reserve"/>
+    <tableColumn id="18" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_Quantity"/>
+    <tableColumn id="19" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_ReservedQtyBase"/>
+    <tableColumn id="20" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_FullyReserved"/>
+    <tableColumn id="21" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_UnitofMeasureCode"/>
+    <tableColumn id="22" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_UnitPriceExcl_VAT"/>
+    <tableColumn id="23" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_UnitCost"/>
+    <tableColumn id="24" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_UnitCost_LCY"/>
+    <tableColumn id="25" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_LineAmountExclVAT"/>
+    <tableColumn id="26" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_LineAmountExclVATLCY"/>
+    <tableColumn id="27" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_ShipmentDate"/>
+    <tableColumn id="28" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_OutstandingQuantity"/>
+    <tableColumn id="29" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_OutstandingQtyBase"/>
+    <tableColumn id="30" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_Calculated"/>
+    <tableColumn id="31" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_CustomerPostingGroup"/>
+    <tableColumn id="32" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_ApprovedQuantity"/>
+    <tableColumn id="33" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_ApprovedUnitPrice"/>
+    <tableColumn id="34" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="SO_ApprovedAmount"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="SalesOrderActual" displayName="SalesOrderActual" ref="A1:X2" totalsRowShown="0" headerRowDxfId="6" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" mc:Ignorable="xr xr3">
-  <x:autoFilter ref="A1:X2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
-  <x:tableColumns count="24">
-    <x:tableColumn id="1" name="ACT_ShipmentDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="2" name="ACT_PostingDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="3" name="ACT_DocumentDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="4" name="ACT_No" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="5" name="ACT_CustomerNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="6" name="ACT_Customer" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="7" name="ACT_OrderNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="8" name="ACT_OEMNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="9" name="ACT_OEMName" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="10" name="ACT_CurrencyCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="11" name="ACT_DueDate" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="12" name="ACT_Amount" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="13" name="ACT_AmountLCY" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="14" name="ACT_AmountIncludingVAT" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="15" name="ACT_ExternalDocumentNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="16" name="ACT_RemainingAmount" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="17" name="ACT_LocationCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="18" name="ACT_PrintedNo" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="19" name="ACT_Closed" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="20" name="ACT_Cancelled" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="21" name="ACT_Corrective" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="22" name="ACT_ShipmentMethodCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="23" name="ACT_CustomerGroupCode" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="24" name="ACT_CustomerPostingGroup" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="SalesOrderActual" displayName="SalesOrderActual" ref="A1:X2" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:X2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
+  <tableColumns count="24">
+    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_ShipmentDate"/>
+    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_PostingDate"/>
+    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_DocumentDate"/>
+    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_No"/>
+    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_CustomerNo"/>
+    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_Customer"/>
+    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_OrderNo"/>
+    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_OEMNo"/>
+    <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_OEMName"/>
+    <tableColumn id="10" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_CurrencyCode"/>
+    <tableColumn id="11" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_DueDate"/>
+    <tableColumn id="12" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_Amount"/>
+    <tableColumn id="13" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_AmountLCY"/>
+    <tableColumn id="14" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_AmountIncludingVAT"/>
+    <tableColumn id="15" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_ExternalDocumentNo"/>
+    <tableColumn id="16" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_RemainingAmount"/>
+    <tableColumn id="17" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_LocationCode"/>
+    <tableColumn id="18" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_PrintedNo"/>
+    <tableColumn id="19" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_Closed"/>
+    <tableColumn id="20" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_Cancelled"/>
+    <tableColumn id="21" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_Corrective"/>
+    <tableColumn id="22" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_ShipmentMethodCode"/>
+    <tableColumn id="23" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_CustomerGroupCode"/>
+    <tableColumn id="24" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="ACT_CustomerPostingGroup"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1602,22 +1668,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2288BB9B-6709-47CB-B7C9-817F1E183987}">
-  <dimension ref="A1:B2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0040663C-C8D4-4D1A-8BDF-B313A5705AB3}">
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="5" t="s">
         <v>64</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="C1" s="5" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="6">
         <f>DateSheet[[#This Row],[From]]</f>
         <v>0</v>
@@ -1625,228 +1695,48 @@
       <c r="B2" s="6">
         <f>DateSheet[[#This Row],[To]]</f>
         <v>0</v>
+      </c>
+      <c r="C2" s="6" t="str">
+        <f>DateSheet[[#This Row],[CustPostGrpFilter]]</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27192392-EA00-44B3-AE44-538F8098BAFA}">
-  <dimension ref="A1:AH2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EEA1F2F-74E0-45C1-906B-77595ED60E81}">
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="18.4140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" t="s">
         <v>66</v>
       </c>
-      <c r="B1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E1" t="s">
-        <v>70</v>
-      </c>
-      <c r="F1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I1" t="s">
-        <v>74</v>
-      </c>
-      <c r="J1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K1" t="s">
-        <v>76</v>
-      </c>
-      <c r="L1" t="s">
-        <v>77</v>
-      </c>
-      <c r="M1" t="s">
-        <v>78</v>
-      </c>
-      <c r="N1" t="s">
-        <v>79</v>
-      </c>
-      <c r="O1" t="s">
-        <v>80</v>
-      </c>
-      <c r="P1" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>82</v>
-      </c>
-      <c r="R1" t="s">
-        <v>83</v>
-      </c>
-      <c r="S1" t="s">
-        <v>84</v>
-      </c>
-      <c r="T1" t="s">
-        <v>85</v>
-      </c>
-      <c r="U1" t="s">
-        <v>86</v>
-      </c>
-      <c r="V1" t="s">
-        <v>87</v>
-      </c>
-      <c r="W1" t="s">
-        <v>88</v>
-      </c>
-      <c r="X1" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>92</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>93</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>94</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>95</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>96</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>97</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B2" t="s">
-        <v>100</v>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D2" t="s">
-        <v>100</v>
-      </c>
-      <c r="E2" t="s">
-        <v>100</v>
-      </c>
-      <c r="F2" t="s">
-        <v>100</v>
-      </c>
-      <c r="G2" t="s">
-        <v>100</v>
-      </c>
-      <c r="H2" t="s">
-        <v>100</v>
-      </c>
-      <c r="I2" t="s">
-        <v>100</v>
-      </c>
-      <c r="J2" t="s">
-        <v>100</v>
-      </c>
-      <c r="K2" s="2">
-        <v>0</v>
-      </c>
-      <c r="L2" s="2">
-        <v>0</v>
-      </c>
-      <c r="M2" s="2">
-        <v>0</v>
-      </c>
-      <c r="N2" t="s">
-        <v>100</v>
-      </c>
-      <c r="O2" t="s">
-        <v>100</v>
-      </c>
-      <c r="P2" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>100</v>
-      </c>
-      <c r="R2" s="3">
-        <v>0</v>
-      </c>
-      <c r="S2" s="3">
-        <v>0</v>
-      </c>
-      <c r="T2" t="s">
-        <v>101</v>
-      </c>
-      <c r="U2" t="s">
-        <v>100</v>
-      </c>
-      <c r="V2" s="3">
-        <v>0</v>
-      </c>
-      <c r="W2" s="3">
-        <v>0</v>
-      </c>
-      <c r="X2" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>100</v>
-      </c>
-      <c r="AF2" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH2" s="3">
-        <v>0</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1859,159 +1749,219 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F92DA9B0-E3EE-41F4-96E1-D3C723C10EF1}">
-  <dimension ref="A1:X2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{981BC914-4D47-4A04-9E35-DFDFDA0D8DD0}">
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="18.4140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" t="s">
+        <v>76</v>
+      </c>
+      <c r="J1" t="s">
+        <v>77</v>
+      </c>
+      <c r="K1" t="s">
+        <v>78</v>
+      </c>
+      <c r="L1" t="s">
+        <v>79</v>
+      </c>
+      <c r="M1" t="s">
+        <v>80</v>
+      </c>
+      <c r="N1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O1" t="s">
+        <v>82</v>
+      </c>
+      <c r="P1" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>84</v>
+      </c>
+      <c r="R1" t="s">
+        <v>85</v>
+      </c>
+      <c r="S1" t="s">
+        <v>86</v>
+      </c>
+      <c r="T1" t="s">
+        <v>87</v>
+      </c>
+      <c r="U1" t="s">
+        <v>88</v>
+      </c>
+      <c r="V1" t="s">
+        <v>89</v>
+      </c>
+      <c r="W1" t="s">
+        <v>90</v>
+      </c>
+      <c r="X1" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>92</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>96</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:34" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I2" t="s">
+        <v>67</v>
+      </c>
+      <c r="J2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0</v>
+      </c>
+      <c r="N2" t="s">
+        <v>67</v>
+      </c>
+      <c r="O2" t="s">
+        <v>67</v>
+      </c>
+      <c r="P2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>67</v>
+      </c>
+      <c r="R2" s="3">
+        <v>0</v>
+      </c>
+      <c r="S2" s="3">
+        <v>0</v>
+      </c>
+      <c r="T2" t="s">
         <v>102</v>
       </c>
-      <c r="B1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1" t="s">
-        <v>106</v>
-      </c>
-      <c r="F1" t="s">
-        <v>107</v>
-      </c>
-      <c r="G1" t="s">
-        <v>108</v>
-      </c>
-      <c r="H1" t="s">
-        <v>109</v>
-      </c>
-      <c r="I1" t="s">
-        <v>110</v>
-      </c>
-      <c r="J1" t="s">
-        <v>111</v>
-      </c>
-      <c r="K1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L1" t="s">
-        <v>113</v>
-      </c>
-      <c r="M1" t="s">
-        <v>114</v>
-      </c>
-      <c r="N1" t="s">
-        <v>115</v>
-      </c>
-      <c r="O1" t="s">
-        <v>116</v>
-      </c>
-      <c r="P1" t="s">
-        <v>117</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>118</v>
-      </c>
-      <c r="R1" t="s">
-        <v>119</v>
-      </c>
-      <c r="S1" t="s">
-        <v>120</v>
-      </c>
-      <c r="T1" t="s">
-        <v>121</v>
-      </c>
-      <c r="U1" t="s">
-        <v>122</v>
-      </c>
-      <c r="V1" t="s">
-        <v>123</v>
-      </c>
-      <c r="W1" t="s">
-        <v>124</v>
-      </c>
-      <c r="X1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="2">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0</v>
-      </c>
-      <c r="D2" t="s">
-        <v>100</v>
-      </c>
-      <c r="E2" t="s">
-        <v>100</v>
-      </c>
-      <c r="F2" t="s">
-        <v>100</v>
-      </c>
-      <c r="G2" t="s">
-        <v>100</v>
-      </c>
-      <c r="H2" t="s">
-        <v>100</v>
-      </c>
-      <c r="I2" t="s">
-        <v>100</v>
-      </c>
-      <c r="J2" t="s">
-        <v>100</v>
-      </c>
-      <c r="K2" s="2">
-        <v>0</v>
-      </c>
-      <c r="L2" s="3">
-        <v>0</v>
-      </c>
-      <c r="M2" s="3">
-        <v>0</v>
-      </c>
-      <c r="N2" s="3">
-        <v>0</v>
-      </c>
-      <c r="O2" t="s">
-        <v>100</v>
-      </c>
-      <c r="P2" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>100</v>
-      </c>
-      <c r="R2" s="4">
-        <v>0</v>
-      </c>
-      <c r="S2" t="s">
-        <v>101</v>
-      </c>
-      <c r="T2" t="s">
-        <v>101</v>
-      </c>
       <c r="U2" t="s">
-        <v>101</v>
-      </c>
-      <c r="V2" t="s">
-        <v>100</v>
-      </c>
-      <c r="W2" t="s">
-        <v>100</v>
-      </c>
-      <c r="X2" t="s">
-        <v>100</v>
+        <v>67</v>
+      </c>
+      <c r="V2" s="3">
+        <v>0</v>
+      </c>
+      <c r="W2" s="3">
+        <v>0</v>
+      </c>
+      <c r="X2" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="2">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2024,7 +1974,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A66A90A-21D5-44F1-8F52-486D346401A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C63C6D6-5D17-40A3-BB33-4E9BDCE20C67}">
   <dimension ref="A1:X2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -2033,76 +1983,76 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H1" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1" t="s">
+        <v>111</v>
+      </c>
+      <c r="J1" t="s">
+        <v>112</v>
+      </c>
+      <c r="K1" t="s">
+        <v>113</v>
+      </c>
+      <c r="L1" t="s">
+        <v>114</v>
+      </c>
+      <c r="M1" t="s">
+        <v>115</v>
+      </c>
+      <c r="N1" t="s">
+        <v>116</v>
+      </c>
+      <c r="O1" t="s">
+        <v>117</v>
+      </c>
+      <c r="P1" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>119</v>
+      </c>
+      <c r="R1" t="s">
+        <v>120</v>
+      </c>
+      <c r="S1" t="s">
+        <v>121</v>
+      </c>
+      <c r="T1" t="s">
+        <v>122</v>
+      </c>
+      <c r="U1" t="s">
+        <v>123</v>
+      </c>
+      <c r="V1" t="s">
+        <v>124</v>
+      </c>
+      <c r="W1" t="s">
+        <v>125</v>
+      </c>
+      <c r="X1" t="s">
         <v>126</v>
-      </c>
-      <c r="B1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F1" t="s">
-        <v>131</v>
-      </c>
-      <c r="G1" t="s">
-        <v>132</v>
-      </c>
-      <c r="H1" t="s">
-        <v>133</v>
-      </c>
-      <c r="I1" t="s">
-        <v>134</v>
-      </c>
-      <c r="J1" t="s">
-        <v>135</v>
-      </c>
-      <c r="K1" t="s">
-        <v>136</v>
-      </c>
-      <c r="L1" t="s">
-        <v>137</v>
-      </c>
-      <c r="M1" t="s">
-        <v>138</v>
-      </c>
-      <c r="N1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O1" t="s">
-        <v>140</v>
-      </c>
-      <c r="P1" t="s">
-        <v>141</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>142</v>
-      </c>
-      <c r="R1" t="s">
-        <v>143</v>
-      </c>
-      <c r="S1" t="s">
-        <v>144</v>
-      </c>
-      <c r="T1" t="s">
-        <v>145</v>
-      </c>
-      <c r="U1" t="s">
-        <v>146</v>
-      </c>
-      <c r="V1" t="s">
-        <v>147</v>
-      </c>
-      <c r="W1" t="s">
-        <v>148</v>
-      </c>
-      <c r="X1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.55000000000000004">
@@ -2116,25 +2066,25 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="G2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="H2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="J2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="K2" s="2">
         <v>0</v>
@@ -2149,34 +2099,34 @@
         <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="P2" s="3">
         <v>0</v>
       </c>
       <c r="Q2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="R2" s="4">
         <v>0</v>
       </c>
       <c r="S2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="U2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="V2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="W2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="X2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -2189,7 +2139,172 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3EE184B-5E4B-4589-AF05-0E22CA869E0C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50EF979F-0B9A-4578-A85F-2D7B01C74680}">
+  <dimension ref="A1:X2"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="18.4140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F1" t="s">
+        <v>132</v>
+      </c>
+      <c r="G1" t="s">
+        <v>133</v>
+      </c>
+      <c r="H1" t="s">
+        <v>134</v>
+      </c>
+      <c r="I1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J1" t="s">
+        <v>136</v>
+      </c>
+      <c r="K1" t="s">
+        <v>137</v>
+      </c>
+      <c r="L1" t="s">
+        <v>138</v>
+      </c>
+      <c r="M1" t="s">
+        <v>139</v>
+      </c>
+      <c r="N1" t="s">
+        <v>140</v>
+      </c>
+      <c r="O1" t="s">
+        <v>141</v>
+      </c>
+      <c r="P1" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>143</v>
+      </c>
+      <c r="R1" t="s">
+        <v>144</v>
+      </c>
+      <c r="S1" t="s">
+        <v>145</v>
+      </c>
+      <c r="T1" t="s">
+        <v>146</v>
+      </c>
+      <c r="U1" t="s">
+        <v>147</v>
+      </c>
+      <c r="V1" t="s">
+        <v>148</v>
+      </c>
+      <c r="W1" t="s">
+        <v>149</v>
+      </c>
+      <c r="X1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I2" t="s">
+        <v>67</v>
+      </c>
+      <c r="J2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" s="3">
+        <v>0</v>
+      </c>
+      <c r="M2" s="3">
+        <v>0</v>
+      </c>
+      <c r="N2" s="3">
+        <v>0</v>
+      </c>
+      <c r="O2" t="s">
+        <v>67</v>
+      </c>
+      <c r="P2" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>67</v>
+      </c>
+      <c r="R2" s="4">
+        <v>0</v>
+      </c>
+      <c r="S2" t="s">
+        <v>102</v>
+      </c>
+      <c r="T2" t="s">
+        <v>102</v>
+      </c>
+      <c r="U2" t="s">
+        <v>102</v>
+      </c>
+      <c r="V2" t="s">
+        <v>67</v>
+      </c>
+      <c r="W2" t="s">
+        <v>67</v>
+      </c>
+      <c r="X2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{430E0508-8182-402C-BB5C-94216E748C4D}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -2198,54 +2313,99 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="G2" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="H2" t="s">
-        <v>100</v>
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{608D0135-2DF7-49FC-B6AE-C7E70BA2A176}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="18.4140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2258,7 +2418,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A35B9210-B6E3-46CF-81BC-9E9F60A92CA5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6165BDF-A7B8-4D4C-8853-4505EFD5181D}">
   <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -2296,106 +2456,106 @@
   <sheetData>
     <row r="1" spans="1:34" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="7" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="Q1" s="7" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="R1" s="7" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="T1" s="7" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="U1" s="7" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="V1" s="7" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="W1" s="7" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="X1" s="7" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="Y1" s="7" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="Z1" s="7" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="AA1" s="7" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="AB1" s="7" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="AC1" s="7" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="AD1" s="7" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="AE1" s="7" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="AF1" s="7" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
       <c r="AG1" s="7" t="s">
-        <v>214</v>
+        <v>195</v>
       </c>
       <c r="AH1" s="7" t="s">
-        <v>215</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.55000000000000004">
@@ -2515,7 +2675,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56840D0B-8804-46AE-B3BE-559BAFBC6888}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725428D0-B942-47B5-9F5D-93EB92F0047F}">
   <dimension ref="A1:X2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -2547,76 +2707,76 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="7" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="G1" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q1" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="T1" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="U1" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="W1" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="X1" s="7" t="s">
         <v>193</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="N1" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="O1" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="P1" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="Q1" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="R1" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="S1" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="T1" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="U1" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="V1" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="W1" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="X1" s="7" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.55000000000000004">
@@ -2706,7 +2866,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1D4F6D3-DFEC-43BB-800E-1779455D7C29}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42C57AD0-3996-4582-818A-70AB431AAF08}">
   <dimension ref="A1:X2"/>
   <sheetFormatPr defaultColWidth="8" defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -2738,76 +2898,76 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="7" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="G1" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q1" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="T1" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="U1" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="W1" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="X1" s="7" t="s">
         <v>193</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="N1" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="O1" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="P1" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="Q1" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="R1" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="S1" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="T1" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="U1" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="V1" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="W1" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="X1" s="7" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.55000000000000004">
@@ -2897,7 +3057,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D2E03B7-FCA7-4FF6-BEA9-3EE78EADAC61}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91F4A507-15D8-4D80-BC26-7A322F37000C}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -2913,28 +3073,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -2976,7 +3136,52 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7C3209-4FB4-46E5-B547-2A4209A8ABCA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D7458BB-6DBE-4223-AA55-988AF8F2F52F}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="2" max="2" width="6.08203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.4140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" t="str" cm="1">
+        <f t="array" ref="A2:D2">OrderSummarybyCustomer[#Data]</f>
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5868C5B5-835D-4709-9822-BD56B4DD3EE2}">
   <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -3004,8 +3209,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{422D5196-3FFF-40B1-8A46-5041F28C8F69}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFEE4FCE-0E93-4DED-82D7-5F91E270A9CE}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -3038,8 +3243,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CD85515-4283-40F5-8591-E930E868C6F6}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A07A0A2-2C54-45E0-8D25-6A8565D8270F}">
   <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -3294,39 +3499,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6BF9F0-EB50-4DC9-A7EE-E7D02518FDBF}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
-  <cols>
-    <col min="1" max="1" width="18.4140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="2">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{f42aa342-8706-4288-bd11-ebb85995028c}" enabled="1" method="Standard" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" contentBits="0" removed="0"/>

</xml_diff>